<commit_message>
:kiwi_fruit: NMDS dataset 1 filtered at 20% with clearer labels
</commit_message>
<xml_diff>
--- a/data/derived_data/4_Diversities/ps_16S_rare_expe_D1_20_tax_table.xlsx
+++ b/data/derived_data/4_Diversities/ps_16S_rare_expe_D1_20_tax_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -104,9 +104,15 @@
     <t xml:space="preserve">Erwiniaceae</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_12</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_1247</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_1247</t>
+  </si>
+  <si>
     <t xml:space="preserve">Acetobacter thailandicus</t>
   </si>
   <si>
@@ -161,9 +167,15 @@
     <t xml:space="preserve">Cluster_1567</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_1567</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_16</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_16</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_17</t>
   </si>
   <si>
@@ -173,9 +185,15 @@
     <t xml:space="preserve">Cluster_18</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_18</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_181</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_181</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_20</t>
   </si>
   <si>
@@ -185,12 +203,18 @@
     <t xml:space="preserve">Cluster_21</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_21</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_22</t>
   </si>
   <si>
     <t xml:space="preserve">Enterobacteriaceae</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_22</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_23</t>
   </si>
   <si>
@@ -248,6 +272,9 @@
     <t xml:space="preserve">Cluster_255</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_255</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_2621</t>
   </si>
   <si>
@@ -257,6 +284,9 @@
     <t xml:space="preserve">Cluster_267</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_267</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_28</t>
   </si>
   <si>
@@ -266,6 +296,9 @@
     <t xml:space="preserve">Rhodanobacteraceae</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_28</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_284</t>
   </si>
   <si>
@@ -299,6 +332,9 @@
     <t xml:space="preserve">Cluster_38</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_38</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_39</t>
   </si>
   <si>
@@ -311,6 +347,9 @@
     <t xml:space="preserve">Cluster_3951</t>
   </si>
   <si>
+    <t xml:space="preserve">Unknown_3951</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cluster_407</t>
   </si>
   <si>
@@ -402,6 +441,9 @@
   </si>
   <si>
     <t xml:space="preserve">Yersiniaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unknown_87</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_9</t>
@@ -863,7 +905,7 @@
         <v>29</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H5" t="s">
         <v>15</v>
@@ -871,7 +913,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
@@ -889,15 +931,15 @@
         <v>20</v>
       </c>
       <c r="G6" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="H6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -909,13 +951,13 @@
         <v>18</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H7" t="s">
         <v>15</v>
@@ -923,7 +965,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -949,7 +991,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
@@ -967,15 +1009,15 @@
         <v>13</v>
       </c>
       <c r="G9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
@@ -993,7 +1035,7 @@
         <v>20</v>
       </c>
       <c r="G10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H10" t="s">
         <v>15</v>
@@ -1001,7 +1043,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
@@ -1013,13 +1055,13 @@
         <v>23</v>
       </c>
       <c r="E11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H11" t="s">
         <v>15</v>
@@ -1027,7 +1069,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B12" t="s">
         <v>9</v>
@@ -1045,7 +1087,7 @@
         <v>20</v>
       </c>
       <c r="G12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H12" t="s">
         <v>15</v>
@@ -1053,7 +1095,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
         <v>9</v>
@@ -1079,7 +1121,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
@@ -1097,7 +1139,7 @@
         <v>29</v>
       </c>
       <c r="G14" t="s">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="H14" t="s">
         <v>15</v>
@@ -1105,7 +1147,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
@@ -1123,7 +1165,7 @@
         <v>29</v>
       </c>
       <c r="G15" t="s">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="H15" t="s">
         <v>15</v>
@@ -1131,7 +1173,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B16" t="s">
         <v>9</v>
@@ -1152,12 +1194,12 @@
         <v>21</v>
       </c>
       <c r="H16" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B17" t="s">
         <v>9</v>
@@ -1175,7 +1217,7 @@
         <v>20</v>
       </c>
       <c r="G17" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="H17" t="s">
         <v>15</v>
@@ -1183,7 +1225,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B18" t="s">
         <v>9</v>
@@ -1201,7 +1243,7 @@
         <v>29</v>
       </c>
       <c r="G18" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="H18" t="s">
         <v>15</v>
@@ -1209,7 +1251,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
         <v>9</v>
@@ -1227,15 +1269,15 @@
         <v>20</v>
       </c>
       <c r="G19" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H19" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B20" t="s">
         <v>9</v>
@@ -1261,7 +1303,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
         <v>9</v>
@@ -1276,10 +1318,10 @@
         <v>28</v>
       </c>
       <c r="F21" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="G21" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="H21" t="s">
         <v>15</v>
@@ -1287,7 +1329,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
@@ -1302,10 +1344,10 @@
         <v>28</v>
       </c>
       <c r="F22" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="G22" t="s">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="H22" t="s">
         <v>15</v>
@@ -1313,7 +1355,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B23" t="s">
         <v>9</v>
@@ -1325,13 +1367,13 @@
         <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="F23" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="G23" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H23" t="s">
         <v>15</v>
@@ -1339,7 +1381,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B24" t="s">
         <v>9</v>
@@ -1351,13 +1393,13 @@
         <v>18</v>
       </c>
       <c r="E24" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="F24" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="G24" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="H24" t="s">
         <v>15</v>
@@ -1365,7 +1407,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B25" t="s">
         <v>9</v>
@@ -1377,13 +1419,13 @@
         <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="F25" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="G25" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H25" t="s">
         <v>15</v>
@@ -1391,25 +1433,25 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="B26" t="s">
         <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="D26" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="E26" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="F26" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G26" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="H26" t="s">
         <v>15</v>
@@ -1417,7 +1459,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="B27" t="s">
         <v>9</v>
@@ -1432,10 +1474,10 @@
         <v>15</v>
       </c>
       <c r="F27" t="s">
-        <v>15</v>
+        <v>86</v>
       </c>
       <c r="G27" t="s">
-        <v>15</v>
+        <v>86</v>
       </c>
       <c r="H27" t="s">
         <v>15</v>
@@ -1443,7 +1485,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="B28" t="s">
         <v>9</v>
@@ -1461,7 +1503,7 @@
         <v>20</v>
       </c>
       <c r="G28" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H28" t="s">
         <v>15</v>
@@ -1469,25 +1511,25 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
+        <v>89</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" t="s">
         <v>80</v>
       </c>
-      <c r="B29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C29" t="s">
-        <v>72</v>
-      </c>
       <c r="D29" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="E29" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="F29" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G29" t="s">
-        <v>15</v>
+        <v>90</v>
       </c>
       <c r="H29" t="s">
         <v>15</v>
@@ -1495,7 +1537,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="B30" t="s">
         <v>9</v>
@@ -1507,13 +1549,13 @@
         <v>23</v>
       </c>
       <c r="E30" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="F30" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G30" t="s">
-        <v>15</v>
+        <v>94</v>
       </c>
       <c r="H30" t="s">
         <v>15</v>
@@ -1521,7 +1563,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="B31" t="s">
         <v>9</v>
@@ -1536,10 +1578,10 @@
         <v>28</v>
       </c>
       <c r="F31" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="G31" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="H31" t="s">
         <v>15</v>
@@ -1547,7 +1589,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="B32" t="s">
         <v>9</v>
@@ -1573,7 +1615,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="B33" t="s">
         <v>9</v>
@@ -1591,7 +1633,7 @@
         <v>20</v>
       </c>
       <c r="G33" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="H33" t="s">
         <v>15</v>
@@ -1599,7 +1641,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="B34" t="s">
         <v>9</v>
@@ -1617,7 +1659,7 @@
         <v>20</v>
       </c>
       <c r="G34" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H34" t="s">
         <v>15</v>
@@ -1625,7 +1667,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="B35" t="s">
         <v>9</v>
@@ -1643,7 +1685,7 @@
         <v>29</v>
       </c>
       <c r="G35" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="H35" t="s">
         <v>15</v>
@@ -1651,7 +1693,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="B36" t="s">
         <v>9</v>
@@ -1669,7 +1711,7 @@
         <v>29</v>
       </c>
       <c r="G36" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="H36" t="s">
         <v>15</v>
@@ -1677,7 +1719,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="B37" t="s">
         <v>9</v>
@@ -1692,10 +1734,10 @@
         <v>15</v>
       </c>
       <c r="F37" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="G37" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="H37" t="s">
         <v>15</v>
@@ -1703,7 +1745,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="B38" t="s">
         <v>9</v>
@@ -1715,13 +1757,13 @@
         <v>23</v>
       </c>
       <c r="E38" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F38" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="G38" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="H38" t="s">
         <v>15</v>
@@ -1729,7 +1771,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="B39" t="s">
         <v>9</v>
@@ -1747,7 +1789,7 @@
         <v>20</v>
       </c>
       <c r="G39" t="s">
-        <v>15</v>
+        <v>111</v>
       </c>
       <c r="H39" t="s">
         <v>15</v>
@@ -1755,25 +1797,25 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="B40" t="s">
         <v>9</v>
       </c>
       <c r="C40" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="D40" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="E40" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="F40" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="G40" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="H40" t="s">
         <v>15</v>
@@ -1781,7 +1823,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="B41" t="s">
         <v>9</v>
@@ -1796,18 +1838,18 @@
         <v>28</v>
       </c>
       <c r="F41" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="G41" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="H41" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="B42" t="s">
         <v>9</v>
@@ -1825,7 +1867,7 @@
         <v>29</v>
       </c>
       <c r="G42" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="H42" t="s">
         <v>15</v>
@@ -1833,7 +1875,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
@@ -1851,15 +1893,15 @@
         <v>20</v>
       </c>
       <c r="G43" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H43" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="B44" t="s">
         <v>9</v>
@@ -1871,13 +1913,13 @@
         <v>11</v>
       </c>
       <c r="E44" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="F44" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="G44" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="H44" t="s">
         <v>15</v>
@@ -1885,7 +1927,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
@@ -1903,7 +1945,7 @@
         <v>13</v>
       </c>
       <c r="G45" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="H45" t="s">
         <v>15</v>
@@ -1911,7 +1953,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
@@ -1932,12 +1974,12 @@
         <v>21</v>
       </c>
       <c r="H46" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
@@ -1949,13 +1991,13 @@
         <v>23</v>
       </c>
       <c r="E47" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F47" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G47" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H47" t="s">
         <v>15</v>
@@ -1963,7 +2005,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="B48" t="s">
         <v>9</v>
@@ -1981,7 +2023,7 @@
         <v>20</v>
       </c>
       <c r="G48" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H48" t="s">
         <v>15</v>
@@ -1989,7 +2031,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>
@@ -2007,7 +2049,7 @@
         <v>20</v>
       </c>
       <c r="G49" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H49" t="s">
         <v>15</v>
@@ -2015,7 +2057,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="B50" t="s">
         <v>9</v>
@@ -2027,13 +2069,13 @@
         <v>18</v>
       </c>
       <c r="E50" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="F50" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="G50" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="H50" t="s">
         <v>15</v>
@@ -2041,7 +2083,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="B51" t="s">
         <v>9</v>
@@ -2059,7 +2101,7 @@
         <v>20</v>
       </c>
       <c r="G51" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H51" t="s">
         <v>15</v>
@@ -2067,7 +2109,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="B52" t="s">
         <v>9</v>
@@ -2079,13 +2121,13 @@
         <v>11</v>
       </c>
       <c r="E52" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="F52" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="G52" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="H52" t="s">
         <v>15</v>
@@ -2093,7 +2135,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="B53" t="s">
         <v>9</v>
@@ -2108,10 +2150,10 @@
         <v>28</v>
       </c>
       <c r="F53" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="G53" t="s">
-        <v>15</v>
+        <v>143</v>
       </c>
       <c r="H53" t="s">
         <v>15</v>
@@ -2119,7 +2161,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="B54" t="s">
         <v>9</v>
@@ -2137,15 +2179,15 @@
         <v>20</v>
       </c>
       <c r="G54" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H54" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B55" t="s">
         <v>9</v>
@@ -2157,13 +2199,13 @@
         <v>11</v>
       </c>
       <c r="E55" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="F55" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="G55" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="H55" t="s">
         <v>15</v>

</xml_diff>